<commit_message>
fix: eBay sync uses actual order fees from API, not 12.35% estimate
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -1240,13 +1240,13 @@
         <v>0.5</v>
       </c>
       <c r="G13" t="n">
-        <v>0.75</v>
+        <v>0.61</v>
       </c>
       <c r="H13" t="n">
         <v>1.11</v>
       </c>
       <c r="I13" t="n">
-        <v>0.25</v>
+        <v>0.11</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -1269,7 +1269,7 @@
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="U13" t="n">
+      <c r="U13" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="G249" s="3" t="n">
-        <v>1339.52</v>
+        <v>1339.38</v>
       </c>
     </row>
     <row r="250">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="I250" s="3" t="n">
-        <v>469.35</v>
+        <v>469.21</v>
       </c>
     </row>
     <row r="251">
@@ -14518,7 +14518,7 @@
         </is>
       </c>
       <c r="I254" s="3" t="n">
-        <v>1217.77</v>
+        <v>1217.63</v>
       </c>
     </row>
   </sheetData>
@@ -14777,7 +14777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14866,6 +14866,29 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-11T19:50:35</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>16</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Special Red Card 82 (Pokemon Chaos Rising)</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Browse by Date uses stored DB values not recalculated fees
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -1296,13 +1296,13 @@
         <v>10</v>
       </c>
       <c r="G14" t="n">
-        <v>16.42</v>
+        <v>16.39</v>
       </c>
       <c r="H14" t="n">
         <v>11</v>
       </c>
       <c r="I14" t="n">
-        <v>6.42</v>
+        <v>6.39</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1325,7 +1325,7 @@
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="U14" t="n">
+      <c r="U14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="G249" s="3" t="n">
-        <v>1339.38</v>
+        <v>1339.35</v>
       </c>
     </row>
     <row r="250">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="I250" s="3" t="n">
-        <v>469.21</v>
+        <v>469.18</v>
       </c>
     </row>
     <row r="251">
@@ -14518,7 +14518,7 @@
         </is>
       </c>
       <c r="I254" s="3" t="n">
-        <v>1217.63</v>
+        <v>1217.6</v>
       </c>
     </row>
   </sheetData>
@@ -14777,7 +14777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14889,6 +14889,29 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-11T19:54:36</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hisuian Zoroark Vstar 62 (Pokemon Japanese Dark Phantasma)</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>16.39</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: store and display actual ebay_fee per sale, item 270 corrected to £0.79
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -1352,13 +1352,13 @@
         <v>17</v>
       </c>
       <c r="G15" t="n">
-        <v>20.16</v>
+        <v>17.88</v>
       </c>
       <c r="H15" t="n">
         <v>31.26</v>
       </c>
       <c r="I15" t="n">
-        <v>3.16</v>
+        <v>0.88</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="U15" t="n">
+      <c r="U15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="G249" s="3" t="n">
-        <v>1339.35</v>
+        <v>1337.07</v>
       </c>
     </row>
     <row r="250">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="I250" s="3" t="n">
-        <v>469.18</v>
+        <v>466.9</v>
       </c>
     </row>
     <row r="251">
@@ -14518,7 +14518,7 @@
         </is>
       </c>
       <c r="I254" s="3" t="n">
-        <v>1217.6</v>
+        <v>1215.32</v>
       </c>
     </row>
   </sheetData>
@@ -14777,7 +14777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14912,6 +14912,29 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-11T19:57:34</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>18</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ho Oh V 140 (Pokemon Silver Tempest)</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: promoted listing % setting, per-item promotion control, auto-apply on eBay listing
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -4714,13 +4714,13 @@
         <v>4</v>
       </c>
       <c r="G76" t="n">
-        <v>4.79</v>
+        <v>4.78</v>
       </c>
       <c r="H76" t="n">
         <v>5.96</v>
       </c>
       <c r="I76" t="n">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
@@ -4743,7 +4743,7 @@
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="U76" t="n">
+      <c r="U76" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="G249" s="3" t="n">
-        <v>1337.07</v>
+        <v>1337.06</v>
       </c>
     </row>
     <row r="250">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="I250" s="3" t="n">
-        <v>466.9</v>
+        <v>466.89</v>
       </c>
     </row>
     <row r="251">
@@ -14518,7 +14518,7 @@
         </is>
       </c>
       <c r="I254" s="3" t="n">
-        <v>1215.32</v>
+        <v>1215.31</v>
       </c>
     </row>
   </sheetData>
@@ -14777,7 +14777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14935,6 +14935,29 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-11T20:06:45</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>148</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Chespin 87 (Pokemon Chaos Rising)</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: apply promotion % to all active eBay listings in one click
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -4770,13 +4770,13 @@
         <v>4</v>
       </c>
       <c r="G77" t="n">
-        <v>2.17</v>
+        <v>1.88</v>
       </c>
       <c r="H77" t="n">
         <v>4.4</v>
       </c>
       <c r="I77" t="n">
-        <v>-1.83</v>
+        <v>-2.12</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
@@ -4791,7 +4791,7 @@
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="U77" t="n">
+      <c r="U77" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="G249" s="3" t="n">
-        <v>1337.06</v>
+        <v>1336.77</v>
       </c>
     </row>
     <row r="250">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="I250" s="3" t="n">
-        <v>466.89</v>
+        <v>466.6</v>
       </c>
     </row>
     <row r="251">
@@ -14518,7 +14518,7 @@
         </is>
       </c>
       <c r="I254" s="3" t="n">
-        <v>1215.31</v>
+        <v>1215.02</v>
       </c>
     </row>
   </sheetData>
@@ -14777,7 +14777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14958,6 +14958,29 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-11T20:09:58</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>149</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mega Greninja Ex 22 (Pokemon Chaos Rising)</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: already listed button to manually sync eBay listing ID
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -7381,13 +7381,13 @@
         <v>0.5</v>
       </c>
       <c r="G120" t="n">
-        <v>0.93</v>
+        <v>0.49</v>
       </c>
       <c r="H120" t="n">
         <v>1.1</v>
       </c>
       <c r="I120" t="n">
-        <v>0.43</v>
+        <v>-0.01</v>
       </c>
       <c r="L120" t="inlineStr">
         <is>
@@ -7402,7 +7402,7 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="U120" t="n">
+      <c r="U120" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7538,10 +7538,10 @@
         <v>20</v>
       </c>
       <c r="G123" t="n">
-        <v>31.47</v>
+        <v>33.26</v>
       </c>
       <c r="I123" t="n">
-        <v>11.47</v>
+        <v>13.26</v>
       </c>
       <c r="L123" t="inlineStr">
         <is>
@@ -7556,7 +7556,7 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="U123" t="n">
+      <c r="U123" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7583,13 +7583,13 @@
         <v>14.49</v>
       </c>
       <c r="G124" t="n">
-        <v>22.39</v>
+        <v>22.34</v>
       </c>
       <c r="H124" t="n">
-        <v>21.11</v>
+        <v>22.4</v>
       </c>
       <c r="I124" t="n">
-        <v>7.9</v>
+        <v>7.85</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
@@ -7604,7 +7604,7 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="U124" t="n">
+      <c r="U124" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7631,13 +7631,13 @@
         <v>12</v>
       </c>
       <c r="G125" t="n">
-        <v>13.57</v>
+        <v>13.49</v>
       </c>
       <c r="H125" t="n">
         <v>13.2</v>
       </c>
       <c r="I125" t="n">
-        <v>1.57</v>
+        <v>1.49</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -7660,7 +7660,7 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="U125" t="n">
+      <c r="U125" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="G249" s="3" t="n">
-        <v>1336.77</v>
+        <v>1337.99</v>
       </c>
     </row>
     <row r="250">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="I250" s="3" t="n">
-        <v>466.6</v>
+        <v>467.82</v>
       </c>
     </row>
     <row r="251">
@@ -14518,7 +14518,7 @@
         </is>
       </c>
       <c r="I254" s="3" t="n">
-        <v>1215.02</v>
+        <v>1216.24</v>
       </c>
     </row>
   </sheetData>
@@ -14777,7 +14777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14981,6 +14981,121 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-11T20:13:03</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>193</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Blaziken 42 (Pokemon Destined Rivals)</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-11T20:17:49</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>196</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Zekrom 10 (Pokemon Celebrations)</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-11T20:28:49</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>199</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Emboar 98 (Pokemon White Flare)</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>33.26</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-11T20:32:47</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>200</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ethan's Typhlosion 190 (Pokemon Destined Rivals)</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>22.34</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-11T20:38:29</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>201</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>M Blastoise Ex 22 (Pokemon Evolutions)</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: syncExistingListing calls correct inventory refresh function
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -7812,13 +7812,13 @@
         <v>12</v>
       </c>
       <c r="G128" t="n">
-        <v>20.49</v>
+        <v>20</v>
       </c>
       <c r="H128" t="n">
         <v>31.71</v>
       </c>
       <c r="I128" t="n">
-        <v>8.49</v>
+        <v>8</v>
       </c>
       <c r="L128" t="inlineStr">
         <is>
@@ -7841,7 +7841,7 @@
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="U128" t="n">
+      <c r="U128" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="G249" s="3" t="n">
-        <v>1337.99</v>
+        <v>1337.5</v>
       </c>
     </row>
     <row r="250">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="I250" s="3" t="n">
-        <v>467.82</v>
+        <v>467.33</v>
       </c>
     </row>
     <row r="251">
@@ -14518,7 +14518,7 @@
         </is>
       </c>
       <c r="I254" s="3" t="n">
-        <v>1216.24</v>
+        <v>1215.75</v>
       </c>
     </row>
   </sheetData>
@@ -14777,7 +14777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15096,6 +15096,29 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-11T20:41:02</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>209</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Lickitung 180 (Pokemon Temporal Forces)</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>20</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: remove unsupported promoted_listing_pct param from eBay listing API call
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -7932,13 +7932,13 @@
         <v>11.9</v>
       </c>
       <c r="G130" t="n">
-        <v>19.78</v>
+        <v>19.74</v>
       </c>
       <c r="H130" t="n">
-        <v>28.33</v>
+        <v>35.62</v>
       </c>
       <c r="I130" t="n">
-        <v>7.88</v>
+        <v>7.84</v>
       </c>
       <c r="L130" t="inlineStr">
         <is>
@@ -7953,7 +7953,7 @@
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="U130" t="n">
+      <c r="U130" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7980,13 +7980,13 @@
         <v>3.4</v>
       </c>
       <c r="G131" t="n">
-        <v>3.74</v>
+        <v>3.72</v>
       </c>
       <c r="H131" t="n">
         <v>5.29</v>
       </c>
       <c r="I131" t="n">
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -8009,7 +8009,7 @@
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="U131" t="n">
+      <c r="U131" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8137,13 +8137,13 @@
         <v>15</v>
       </c>
       <c r="G134" t="n">
-        <v>13.62</v>
+        <v>13.39</v>
       </c>
       <c r="H134" t="n">
         <v>20.15</v>
       </c>
       <c r="I134" t="n">
-        <v>-1.38</v>
+        <v>-1.61</v>
       </c>
       <c r="L134" t="inlineStr">
         <is>
@@ -8158,7 +8158,7 @@
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="U134" t="n">
+      <c r="U134" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="G249" s="3" t="n">
-        <v>1337.5</v>
+        <v>1337.21</v>
       </c>
     </row>
     <row r="250">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="I250" s="3" t="n">
-        <v>467.33</v>
+        <v>467.04</v>
       </c>
     </row>
     <row r="251">
@@ -14518,7 +14518,7 @@
         </is>
       </c>
       <c r="I254" s="3" t="n">
-        <v>1215.75</v>
+        <v>1215.46</v>
       </c>
     </row>
   </sheetData>
@@ -14777,7 +14777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15119,6 +15119,75 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-11T20:46:30</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>211</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Reshiram &amp; Charizard Gx 20 (Pokemon World Championships 2019)</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>19.74</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-11T20:49:29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>212</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Tyrunt 70 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-11T20:52:34</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>214</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Reshiram 113 (Pokemon Celebrations)</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>13.39</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: add ebay policies debug endpoint
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -8438,13 +8438,13 @@
         <v>2</v>
       </c>
       <c r="G140" t="n">
-        <v>3.09</v>
+        <v>3.23</v>
       </c>
       <c r="H140" t="n">
         <v>2.9</v>
       </c>
       <c r="I140" t="n">
-        <v>1.09</v>
+        <v>1.23</v>
       </c>
       <c r="L140" t="inlineStr">
         <is>
@@ -8459,7 +8459,7 @@
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="U140" t="n">
+      <c r="U140" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8486,13 +8486,13 @@
         <v>2</v>
       </c>
       <c r="G141" t="n">
-        <v>3.09</v>
+        <v>3.23</v>
       </c>
       <c r="H141" t="n">
         <v>2.9</v>
       </c>
       <c r="I141" t="n">
-        <v>1.09</v>
+        <v>1.23</v>
       </c>
       <c r="L141" t="inlineStr">
         <is>
@@ -8507,7 +8507,7 @@
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="U141" t="n">
+      <c r="U141" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8534,13 +8534,13 @@
         <v>1</v>
       </c>
       <c r="G142" t="n">
-        <v>1.43</v>
+        <v>1.37</v>
       </c>
       <c r="H142" t="n">
         <v>1.82</v>
       </c>
       <c r="I142" t="n">
-        <v>0.43</v>
+        <v>0.37</v>
       </c>
       <c r="L142" t="inlineStr">
         <is>
@@ -8563,7 +8563,7 @@
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="U142" t="n">
+      <c r="U142" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8590,13 +8590,13 @@
         <v>1</v>
       </c>
       <c r="G143" t="n">
-        <v>2.43</v>
+        <v>2.42</v>
       </c>
       <c r="H143" t="n">
         <v>39.19</v>
       </c>
       <c r="I143" t="n">
-        <v>1.43</v>
+        <v>1.42</v>
       </c>
       <c r="L143" t="inlineStr">
         <is>
@@ -8619,7 +8619,7 @@
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="U143" t="n">
+      <c r="U143" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8646,13 +8646,13 @@
         <v>0</v>
       </c>
       <c r="G144" t="n">
-        <v>7.19</v>
+        <v>7.45</v>
       </c>
       <c r="H144" t="n">
         <v>9.5</v>
       </c>
       <c r="I144" t="n">
-        <v>7.19</v>
+        <v>7.45</v>
       </c>
       <c r="L144" t="inlineStr">
         <is>
@@ -8667,7 +8667,7 @@
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="U144" t="n">
+      <c r="U144" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8694,13 +8694,13 @@
         <v>0</v>
       </c>
       <c r="G145" t="n">
-        <v>7.19</v>
+        <v>7.45</v>
       </c>
       <c r="H145" t="n">
         <v>9.5</v>
       </c>
       <c r="I145" t="n">
-        <v>7.19</v>
+        <v>7.45</v>
       </c>
       <c r="L145" t="inlineStr">
         <is>
@@ -8715,7 +8715,7 @@
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="U145" t="n">
+      <c r="U145" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8790,13 +8790,13 @@
         <v>0</v>
       </c>
       <c r="G147" t="n">
-        <v>7.21</v>
+        <v>7.45</v>
       </c>
       <c r="H147" t="n">
         <v>9.5</v>
       </c>
       <c r="I147" t="n">
-        <v>7.21</v>
+        <v>7.45</v>
       </c>
       <c r="L147" t="inlineStr">
         <is>
@@ -8811,7 +8811,7 @@
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="U147" t="n">
+      <c r="U147" t="b">
         <v>0</v>
       </c>
     </row>
@@ -8838,13 +8838,13 @@
         <v>0</v>
       </c>
       <c r="G148" t="n">
-        <v>7.21</v>
+        <v>7.45</v>
       </c>
       <c r="H148" t="n">
         <v>9.5</v>
       </c>
       <c r="I148" t="n">
-        <v>7.21</v>
+        <v>7.45</v>
       </c>
       <c r="L148" t="inlineStr">
         <is>
@@ -8859,7 +8859,7 @@
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="U148" t="n">
+      <c r="U148" t="b">
         <v>0</v>
       </c>
     </row>
@@ -9204,13 +9204,13 @@
         <v>28</v>
       </c>
       <c r="G155" t="n">
-        <v>35.8</v>
+        <v>42.88</v>
       </c>
       <c r="H155" t="n">
         <v>30.8</v>
       </c>
       <c r="I155" t="n">
-        <v>7.8</v>
+        <v>14.88</v>
       </c>
       <c r="L155" t="inlineStr">
         <is>
@@ -9233,7 +9233,7 @@
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="U155" t="n">
+      <c r="U155" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="G249" s="3" t="n">
-        <v>1337.57</v>
+        <v>1345.86</v>
       </c>
     </row>
     <row r="250">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="I250" s="3" t="n">
-        <v>467.4</v>
+        <v>475.69</v>
       </c>
     </row>
     <row r="251">
@@ -14518,7 +14518,7 @@
         </is>
       </c>
       <c r="I254" s="3" t="n">
-        <v>1215.82</v>
+        <v>1224.11</v>
       </c>
     </row>
   </sheetData>
@@ -14777,7 +14777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15280,6 +15280,213 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-11T21:12:09</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>220</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Hydrapple Cosmos Holo 18 (Pokemon Destined Rivals)</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-11T21:16:29</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>221</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Hydrapple Cosmos Holo 18 (Pokemon Destined Rivals)</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-11T21:19:13</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>222</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Oricorio Ex 110 (Pokemon Phantasmal Flames)</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-11T21:23:07</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>223</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Yamper 99 (Pokemon Phantasmal Flames)</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-11T21:26:05</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>224</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Pikachu World Championships 225 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-11T21:29:30</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>225</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Pikachu World Championships 225 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-11T21:38:43</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>227</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Pikachu World Championships 225 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-11T21:43:26</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>228</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Pikachu World Championships 225 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-11T21:47:21</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>235</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Gyarados Gx 112 (Pokemon Crimson Invasion)</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>42.88</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: move eBay policy IDs to user_profiles, add policy selector in Settings
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -9260,10 +9260,10 @@
         <v>10</v>
       </c>
       <c r="G156" t="n">
-        <v>17.84</v>
+        <v>19.34</v>
       </c>
       <c r="I156" t="n">
-        <v>7.84</v>
+        <v>9.34</v>
       </c>
       <c r="L156" t="inlineStr">
         <is>
@@ -9286,7 +9286,7 @@
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="U156" t="n">
+      <c r="U156" t="b">
         <v>0</v>
       </c>
     </row>
@@ -9478,13 +9478,13 @@
         <v>45</v>
       </c>
       <c r="G160" t="n">
-        <v>52.93</v>
+        <v>52.82</v>
       </c>
       <c r="H160" t="n">
         <v>49.5</v>
       </c>
       <c r="I160" t="n">
-        <v>7.93</v>
+        <v>7.82</v>
       </c>
       <c r="L160" t="inlineStr">
         <is>
@@ -9507,7 +9507,7 @@
           <t>2026-06-10</t>
         </is>
       </c>
-      <c r="U160" t="n">
+      <c r="U160" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10113,10 +10113,10 @@
         <v>1</v>
       </c>
       <c r="G171" t="n">
-        <v>1.49</v>
+        <v>1.48</v>
       </c>
       <c r="I171" t="n">
-        <v>0.49</v>
+        <v>0.48</v>
       </c>
       <c r="L171" t="inlineStr">
         <is>
@@ -10131,7 +10131,7 @@
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="U171" t="n">
+      <c r="U171" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10286,13 +10286,13 @@
         <v>4</v>
       </c>
       <c r="G174" t="n">
-        <v>25.27</v>
+        <v>24.48</v>
       </c>
       <c r="H174" t="n">
-        <v>21.37</v>
+        <v>22.8</v>
       </c>
       <c r="I174" t="n">
-        <v>21.27</v>
+        <v>20.48</v>
       </c>
       <c r="L174" t="inlineStr">
         <is>
@@ -10307,7 +10307,7 @@
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="U174" t="n">
+      <c r="U174" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10334,13 +10334,13 @@
         <v>9</v>
       </c>
       <c r="G175" t="n">
-        <v>4.6</v>
+        <v>4.46</v>
       </c>
       <c r="H175" t="n">
         <v>9.9</v>
       </c>
       <c r="I175" t="n">
-        <v>-4.4</v>
+        <v>-4.54</v>
       </c>
       <c r="L175" t="inlineStr">
         <is>
@@ -10355,7 +10355,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U175" t="n">
+      <c r="U175" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10382,10 +10382,10 @@
         <v>37.64</v>
       </c>
       <c r="G176" t="n">
-        <v>52.26</v>
+        <v>58.03</v>
       </c>
       <c r="I176" t="n">
-        <v>14.62</v>
+        <v>20.39</v>
       </c>
       <c r="L176" t="inlineStr">
         <is>
@@ -10400,7 +10400,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U176" t="n">
+      <c r="U176" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10552,13 +10552,13 @@
         <v>2.77</v>
       </c>
       <c r="G179" t="n">
-        <v>1.59</v>
+        <v>1.48</v>
       </c>
       <c r="H179" t="n">
         <v>3.05</v>
       </c>
       <c r="I179" t="n">
-        <v>-1.18</v>
+        <v>-1.29</v>
       </c>
       <c r="L179" t="inlineStr">
         <is>
@@ -10581,7 +10581,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U179" t="n">
+      <c r="U179" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10672,13 +10672,13 @@
         <v>19.79</v>
       </c>
       <c r="G181" t="n">
-        <v>24.07</v>
+        <v>24.32</v>
       </c>
       <c r="H181" t="n">
         <v>21.77</v>
       </c>
       <c r="I181" t="n">
-        <v>4.28</v>
+        <v>4.53</v>
       </c>
       <c r="L181" t="inlineStr">
         <is>
@@ -10693,7 +10693,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U181" t="n">
+      <c r="U181" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10720,13 +10720,13 @@
         <v>8</v>
       </c>
       <c r="G182" t="n">
-        <v>11.12</v>
+        <v>11.09</v>
       </c>
       <c r="H182" t="n">
         <v>8.800000000000001</v>
       </c>
       <c r="I182" t="n">
-        <v>3.12</v>
+        <v>3.09</v>
       </c>
       <c r="L182" t="inlineStr">
         <is>
@@ -10741,7 +10741,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U182" t="n">
+      <c r="U182" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10768,13 +10768,13 @@
         <v>8</v>
       </c>
       <c r="G183" t="n">
-        <v>11.46</v>
+        <v>11.44</v>
       </c>
       <c r="H183" t="n">
         <v>8.800000000000001</v>
       </c>
       <c r="I183" t="n">
-        <v>3.46</v>
+        <v>3.44</v>
       </c>
       <c r="L183" t="inlineStr">
         <is>
@@ -10789,7 +10789,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U183" t="n">
+      <c r="U183" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10816,13 +10816,13 @@
         <v>16.39</v>
       </c>
       <c r="G184" t="n">
-        <v>36.27</v>
+        <v>36.2</v>
       </c>
       <c r="H184" t="n">
         <v>18.03</v>
       </c>
       <c r="I184" t="n">
-        <v>19.88</v>
+        <v>19.81</v>
       </c>
       <c r="L184" t="inlineStr">
         <is>
@@ -10837,7 +10837,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U184" t="n">
+      <c r="U184" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10864,13 +10864,13 @@
         <v>18</v>
       </c>
       <c r="G185" t="n">
-        <v>32.41</v>
+        <v>32.35</v>
       </c>
       <c r="H185" t="n">
         <v>25.36</v>
       </c>
       <c r="I185" t="n">
-        <v>14.41</v>
+        <v>14.35</v>
       </c>
       <c r="L185" t="inlineStr">
         <is>
@@ -10885,7 +10885,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U185" t="n">
+      <c r="U185" t="b">
         <v>0</v>
       </c>
     </row>
@@ -10912,13 +10912,13 @@
         <v>18</v>
       </c>
       <c r="G186" t="n">
-        <v>29.74</v>
+        <v>29.85</v>
       </c>
       <c r="H186" t="n">
-        <v>28.2</v>
+        <v>27.92</v>
       </c>
       <c r="I186" t="n">
-        <v>11.74</v>
+        <v>11.85</v>
       </c>
       <c r="L186" t="inlineStr">
         <is>
@@ -10933,7 +10933,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U186" t="n">
+      <c r="U186" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11021,13 +11021,13 @@
         <v>15</v>
       </c>
       <c r="G188" t="n">
-        <v>20.93</v>
+        <v>21.46</v>
       </c>
       <c r="H188" t="n">
         <v>24.75</v>
       </c>
       <c r="I188" t="n">
-        <v>5.93</v>
+        <v>6.46</v>
       </c>
       <c r="L188" t="inlineStr">
         <is>
@@ -11042,7 +11042,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U188" t="n">
+      <c r="U188" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11133,13 +11133,13 @@
         <v>4</v>
       </c>
       <c r="G190" t="n">
-        <v>6.07</v>
+        <v>6.03</v>
       </c>
       <c r="H190" t="n">
         <v>7.21</v>
       </c>
       <c r="I190" t="n">
-        <v>2.07</v>
+        <v>2.03</v>
       </c>
       <c r="J190" t="n">
         <v>7.65</v>
@@ -11165,7 +11165,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U190" t="n">
+      <c r="U190" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11192,13 +11192,13 @@
         <v>24.29</v>
       </c>
       <c r="G191" t="n">
-        <v>44.42</v>
+        <v>42.09</v>
       </c>
       <c r="H191" t="n">
-        <v>33.26</v>
+        <v>33.27</v>
       </c>
       <c r="I191" t="n">
-        <v>20.13</v>
+        <v>17.8</v>
       </c>
       <c r="J191" t="n">
         <v>26.72</v>
@@ -11224,7 +11224,7 @@
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="U191" t="n">
+      <c r="U191" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11251,13 +11251,13 @@
         <v>7</v>
       </c>
       <c r="G192" t="n">
-        <v>8.880000000000001</v>
+        <v>7.99</v>
       </c>
       <c r="H192" t="n">
         <v>7.7</v>
       </c>
       <c r="I192" t="n">
-        <v>1.88</v>
+        <v>0.99</v>
       </c>
       <c r="L192" t="inlineStr">
         <is>
@@ -11280,7 +11280,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U192" t="n">
+      <c r="U192" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11307,13 +11307,13 @@
         <v>13</v>
       </c>
       <c r="G193" t="n">
-        <v>20.9</v>
+        <v>22.35</v>
       </c>
       <c r="H193" t="n">
-        <v>18.95</v>
+        <v>18.99</v>
       </c>
       <c r="I193" t="n">
-        <v>7.9</v>
+        <v>9.35</v>
       </c>
       <c r="L193" t="inlineStr">
         <is>
@@ -11336,7 +11336,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U193" t="n">
+      <c r="U193" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11419,13 +11419,13 @@
         <v>1</v>
       </c>
       <c r="G195" t="n">
-        <v>1.12</v>
+        <v>0.96</v>
       </c>
       <c r="H195" t="n">
         <v>1.89</v>
       </c>
       <c r="I195" t="n">
-        <v>0.12</v>
+        <v>-0.04</v>
       </c>
       <c r="L195" t="inlineStr">
         <is>
@@ -11448,7 +11448,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U195" t="n">
+      <c r="U195" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11595,13 +11595,13 @@
         <v>4</v>
       </c>
       <c r="G198" t="n">
-        <v>3.92</v>
+        <v>3.91</v>
       </c>
       <c r="H198" t="n">
-        <v>4.95</v>
+        <v>5.01</v>
       </c>
       <c r="I198" t="n">
-        <v>-0.08</v>
+        <v>-0.09</v>
       </c>
       <c r="L198" t="inlineStr">
         <is>
@@ -11624,7 +11624,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U198" t="n">
+      <c r="U198" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11651,13 +11651,13 @@
         <v>6</v>
       </c>
       <c r="G199" t="n">
-        <v>22.59</v>
+        <v>22.54</v>
       </c>
       <c r="H199" t="n">
-        <v>106.6</v>
+        <v>32.01</v>
       </c>
       <c r="I199" t="n">
-        <v>16.59</v>
+        <v>16.54</v>
       </c>
       <c r="J199" t="n">
         <v>23.82</v>
@@ -11683,7 +11683,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U199" t="n">
+      <c r="U199" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11769,13 +11769,13 @@
         <v>6</v>
       </c>
       <c r="G201" t="n">
-        <v>31.91</v>
+        <v>32.1</v>
       </c>
       <c r="H201" t="n">
-        <v>106.6</v>
+        <v>40.74</v>
       </c>
       <c r="I201" t="n">
-        <v>25.91</v>
+        <v>26.1</v>
       </c>
       <c r="J201" t="n">
         <v>31.69</v>
@@ -11801,7 +11801,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U201" t="n">
+      <c r="U201" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11828,13 +11828,13 @@
         <v>6</v>
       </c>
       <c r="G202" t="n">
-        <v>31.91</v>
+        <v>32.1</v>
       </c>
       <c r="H202" t="n">
-        <v>106.6</v>
+        <v>40.74</v>
       </c>
       <c r="I202" t="n">
-        <v>25.91</v>
+        <v>26.1</v>
       </c>
       <c r="J202" t="n">
         <v>43.94</v>
@@ -11860,7 +11860,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U202" t="n">
+      <c r="U202" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11887,13 +11887,13 @@
         <v>6</v>
       </c>
       <c r="G203" t="n">
-        <v>23.43</v>
+        <v>22.34</v>
       </c>
       <c r="H203" t="n">
         <v>106.6</v>
       </c>
       <c r="I203" t="n">
-        <v>17.43</v>
+        <v>16.34</v>
       </c>
       <c r="J203" t="n">
         <v>23.82</v>
@@ -11919,7 +11919,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U203" t="n">
+      <c r="U203" t="b">
         <v>0</v>
       </c>
     </row>
@@ -11946,13 +11946,13 @@
         <v>6</v>
       </c>
       <c r="G204" t="n">
-        <v>23.43</v>
+        <v>22.34</v>
       </c>
       <c r="H204" t="n">
         <v>106.6</v>
       </c>
       <c r="I204" t="n">
-        <v>17.43</v>
+        <v>16.34</v>
       </c>
       <c r="J204" t="n">
         <v>33.03</v>
@@ -11978,7 +11978,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U204" t="n">
+      <c r="U204" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12248,13 +12248,13 @@
         <v>6</v>
       </c>
       <c r="G209" t="n">
-        <v>5.6</v>
+        <v>5.59</v>
       </c>
       <c r="H209" t="n">
         <v>8.4</v>
       </c>
       <c r="I209" t="n">
-        <v>-0.4</v>
+        <v>-0.41</v>
       </c>
       <c r="J209" t="n">
         <v>10.57</v>
@@ -12280,7 +12280,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U209" t="n">
+      <c r="U209" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12307,13 +12307,13 @@
         <v>4</v>
       </c>
       <c r="G210" t="n">
-        <v>4.48</v>
+        <v>4.47</v>
       </c>
       <c r="H210" t="n">
         <v>31.26</v>
       </c>
       <c r="I210" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="J210" t="n">
         <v>8.84</v>
@@ -12339,7 +12339,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U210" t="n">
+      <c r="U210" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12558,13 +12558,13 @@
         <v>6</v>
       </c>
       <c r="G214" t="n">
-        <v>10.76</v>
+        <v>10.95</v>
       </c>
       <c r="H214" t="n">
         <v>30.62</v>
       </c>
       <c r="I214" t="n">
-        <v>4.76</v>
+        <v>4.95</v>
       </c>
       <c r="J214" t="n">
         <v>14.33</v>
@@ -12590,7 +12590,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U214" t="n">
+      <c r="U214" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12681,13 +12681,13 @@
         <v>6</v>
       </c>
       <c r="G216" t="n">
-        <v>10.76</v>
+        <v>10.95</v>
       </c>
       <c r="H216" t="n">
         <v>30.62</v>
       </c>
       <c r="I216" t="n">
-        <v>4.76</v>
+        <v>4.95</v>
       </c>
       <c r="J216" t="n">
         <v>14.33</v>
@@ -12713,7 +12713,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U216" t="n">
+      <c r="U216" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12740,13 +12740,13 @@
         <v>6</v>
       </c>
       <c r="G217" t="n">
-        <v>10.76</v>
+        <v>10.95</v>
       </c>
       <c r="H217" t="n">
         <v>30.62</v>
       </c>
       <c r="I217" t="n">
-        <v>4.76</v>
+        <v>4.95</v>
       </c>
       <c r="J217" t="n">
         <v>14.33</v>
@@ -12764,7 +12764,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U217" t="n">
+      <c r="U217" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12850,13 +12850,13 @@
         <v>6</v>
       </c>
       <c r="G219" t="n">
-        <v>5.96</v>
+        <v>5.95</v>
       </c>
       <c r="H219" t="n">
         <v>30.62</v>
       </c>
       <c r="I219" t="n">
-        <v>-0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="J219" t="n">
         <v>7.79</v>
@@ -12882,7 +12882,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U219" t="n">
+      <c r="U219" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13024,13 +13024,13 @@
         <v>6</v>
       </c>
       <c r="G222" t="n">
-        <v>6</v>
+        <v>5.99</v>
       </c>
       <c r="H222" t="n">
         <v>30.62</v>
       </c>
       <c r="I222" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="J222" t="n">
         <v>7.88</v>
@@ -13056,7 +13056,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U222" t="n">
+      <c r="U222" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13083,13 +13083,13 @@
         <v>6</v>
       </c>
       <c r="G223" t="n">
-        <v>5.96</v>
+        <v>5.95</v>
       </c>
       <c r="H223" t="n">
         <v>30.62</v>
       </c>
       <c r="I223" t="n">
-        <v>-0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="J223" t="n">
         <v>7.79</v>
@@ -13115,7 +13115,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U223" t="n">
+      <c r="U223" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13206,13 +13206,13 @@
         <v>6</v>
       </c>
       <c r="G225" t="n">
-        <v>5.96</v>
+        <v>5.95</v>
       </c>
       <c r="H225" t="n">
         <v>30.62</v>
       </c>
       <c r="I225" t="n">
-        <v>-0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="J225" t="n">
         <v>7.79</v>
@@ -13238,7 +13238,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U225" t="n">
+      <c r="U225" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13324,13 +13324,13 @@
         <v>6</v>
       </c>
       <c r="G227" t="n">
-        <v>5.96</v>
+        <v>5.95</v>
       </c>
       <c r="H227" t="n">
         <v>30.62</v>
       </c>
       <c r="I227" t="n">
-        <v>-0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="J227" t="n">
         <v>10.57</v>
@@ -13356,7 +13356,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U227" t="n">
+      <c r="U227" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13383,13 +13383,13 @@
         <v>6</v>
       </c>
       <c r="G228" t="n">
-        <v>5.96</v>
+        <v>5.95</v>
       </c>
       <c r="H228" t="n">
         <v>30.62</v>
       </c>
       <c r="I228" t="n">
-        <v>-0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="J228" t="n">
         <v>0</v>
@@ -13415,7 +13415,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U228" t="n">
+      <c r="U228" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13442,13 +13442,13 @@
         <v>6</v>
       </c>
       <c r="G229" t="n">
-        <v>6</v>
+        <v>5.99</v>
       </c>
       <c r="H229" t="n">
         <v>30.62</v>
       </c>
       <c r="I229" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="J229" t="n">
         <v>7.88</v>
@@ -13474,7 +13474,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U229" t="n">
+      <c r="U229" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13501,13 +13501,13 @@
         <v>6</v>
       </c>
       <c r="G230" t="n">
-        <v>6</v>
+        <v>5.99</v>
       </c>
       <c r="H230" t="n">
         <v>30.62</v>
       </c>
       <c r="I230" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="J230" t="n">
         <v>0</v>
@@ -13533,7 +13533,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U230" t="n">
+      <c r="U230" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13560,13 +13560,13 @@
         <v>6</v>
       </c>
       <c r="G231" t="n">
-        <v>6</v>
+        <v>5.99</v>
       </c>
       <c r="H231" t="n">
-        <v>9.75</v>
+        <v>9.24</v>
       </c>
       <c r="I231" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="J231" t="n">
         <v>30</v>
@@ -13592,7 +13592,7 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="U231" t="n">
+      <c r="U231" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13779,13 +13779,13 @@
         <v>1.5</v>
       </c>
       <c r="G235" t="n">
-        <v>1.59</v>
+        <v>1.8</v>
       </c>
       <c r="H235" t="n">
         <v>1.65</v>
       </c>
       <c r="I235" t="n">
-        <v>0.09</v>
+        <v>0.3</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -13800,7 +13800,7 @@
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="U235" t="n">
+      <c r="U235" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13875,13 +13875,13 @@
         <v>3</v>
       </c>
       <c r="G237" t="n">
-        <v>4.11</v>
+        <v>3.43</v>
       </c>
       <c r="H237" t="n">
-        <v>5.14</v>
+        <v>4.99</v>
       </c>
       <c r="I237" t="n">
-        <v>1.11</v>
+        <v>0.43</v>
       </c>
       <c r="L237" t="inlineStr">
         <is>
@@ -13896,7 +13896,7 @@
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="U237" t="n">
+      <c r="U237" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13923,13 +13923,13 @@
         <v>10</v>
       </c>
       <c r="G238" t="n">
-        <v>10.41</v>
+        <v>8.91</v>
       </c>
       <c r="H238" t="n">
         <v>11</v>
       </c>
       <c r="I238" t="n">
-        <v>0.41</v>
+        <v>-1.09</v>
       </c>
       <c r="L238" t="inlineStr">
         <is>
@@ -13944,7 +13944,7 @@
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="U238" t="n">
+      <c r="U238" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14341,13 +14341,13 @@
         <v>6</v>
       </c>
       <c r="G245" t="n">
-        <v>11.76</v>
+        <v>11.91</v>
       </c>
       <c r="H245" t="n">
-        <v>12.34</v>
+        <v>12.29</v>
       </c>
       <c r="I245" t="n">
-        <v>5.76</v>
+        <v>5.91</v>
       </c>
       <c r="J245" t="n">
         <v>13.4</v>
@@ -14373,7 +14373,7 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="U245" t="n">
+      <c r="U245" t="b">
         <v>0</v>
       </c>
       <c r="V245" t="inlineStr">
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="G249" s="3" t="n">
-        <v>1345.86</v>
+        <v>1347.49</v>
       </c>
     </row>
     <row r="250">
@@ -14478,7 +14478,7 @@
         </is>
       </c>
       <c r="I250" s="3" t="n">
-        <v>475.69</v>
+        <v>477.32</v>
       </c>
     </row>
     <row r="251">
@@ -14518,7 +14518,7 @@
         </is>
       </c>
       <c r="I254" s="3" t="n">
-        <v>1224.11</v>
+        <v>1225.74</v>
       </c>
     </row>
   </sheetData>
@@ -14777,7 +14777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15487,6 +15487,1064 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-11T21:53:27</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>236</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Venusaur Vmax Swsh102 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>19.34</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-11T22:00:26</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>269</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Zekrom 114 (Pokemon Black &amp; White)</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>52.82</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-11T22:20:21</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>297</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Paldean Wooper 41 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-11T22:22:33</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>300</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Mega Charizard X Ex 109 (Pokemon Phantasmal Flames)</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>24.48</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-11T22:28:21</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>301</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Mega Scrafty Ex 270 (Pokemon Ascended Heroes)</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07-11T22:35:17</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>302</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Reshiram Rc22 (Pokemon Legendary Treasures)</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>58.03</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-11T22:39:21</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>305</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Drapion 97 (Pokemon Perfect Order)</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-11T22:45:08</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>307</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Reshiram Gx 65 (Pokemon Dragon Majesty)</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>24.32</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-11T22:48:19</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>308</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Gardevoir Gx 140 (Pokemon Burning Shadows)</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-11T22:55:01</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>309</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Ho Oh Gx 131 (Pokemon Burning Shadows)</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-11T22:57:34</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>310</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Sylveon Gx 140 (Pokemon Guardians Rising)</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-11T23:04:13</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>311</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Fennekin Pokemon Center 80 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>32.35</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-11T23:06:49</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>312</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Umbreon Ex 176 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>29.85</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-11T23:11:44</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>314</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Eevee Ex 174 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>21.46</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-11T23:15:27</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>316</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Kartana GX SV73 (Pokemon Hidden Fates)</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-11T23:17:39</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>317</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Gengar Ex 193 (Pokemon Temporal Forces)</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>42.09</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-11T23:21:13</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>318</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Blaziken Cosmos Holo 42 (Pokemon Destined Rivals)</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-11T23:26:35</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>319</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Rayquaza Vmax Tg29 (Pokemon Silver Tempest)</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>22.35</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-07-11T23:33:45</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>321</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Ruffian 181 (Pokemon Journey Together)</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-07-11T23:44:56</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>324</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Lillie's Ribombee 164 (Pokemon Journey Together)</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-07-11T23:49:12</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>325</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Squirtle 39 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>22.54</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-07-11T23:57:29</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>327</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Charmander 38 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-07-12T00:02:29</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>328</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Charmander 38 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-07-12T00:07:50</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>329</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Bulbasaur 37 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>22.34</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-07-12T00:10:30</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>330</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Bulbasaur 37 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>22.34</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-07-12T00:18:52</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>335</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Rowlet 43 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-07-12T00:23:39</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>336</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Popplio 45 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-07-12T00:26:34</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>340</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Piplup 42 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-07-12T00:28:43</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>342</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Piplup 42 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-07-12T00:32:02</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>343</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Piplup 42 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-07-12T00:44:50</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>345</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Chimchar 41 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-07-12T00:52:38</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>348</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Turtwig 40 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-07-12T00:59:38</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>349</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Chimchar 41 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:03:41</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>351</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Chimchar 41 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:11:47</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>353</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Chimchar 41 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:17:24</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>354</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Chimchar 41 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:23:54</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>355</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Turtwig 40 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:27:59</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>356</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Turtwig 40 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:31:17</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>357</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Turtwig #40 Pokemon Promo</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:34:14</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>370</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Mega Feraligatr Ex Jumbo 36 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:36:47</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>371</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Mega Feraligatr Ex Jumbo 36 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:40:13</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>372</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Mega Meganium Ex Jumbo 34 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:42:27</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>373</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Mega Emboar Ex Jumbo 35 (Pokemon Promo)</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:45:03</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>381</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Mega Dragonite Ex 152 (Pokemon Ascended Heroes)</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-07-12T01:47:52</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>383</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Mega Froslass Ex 265 (Pokemon Ascended Heroes)</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-07-12T02:10:58</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>391</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Charmander 1 (Pokemon Tcg Classic Charizard Deck)</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>pricecharting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>